<commit_message>
Add Graphics and diagram
</commit_message>
<xml_diff>
--- a/Workshop-No1/analysis-scripts/titan-plaza-analysis.xlsx
+++ b/Workshop-No1/analysis-scripts/titan-plaza-analysis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8d174e9241cebbab/Documentos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{01281E07-0171-48BC-82CF-A622A6C4782B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="8_{01281E07-0171-48BC-82CF-A622A6C4782B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7C1986A0-565C-4A5F-9A3B-421896147762}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="3" xr2:uid="{A250AC5A-0B7A-4FD7-AD9F-EC65DF86CE1A}"/>
   </bookViews>
@@ -532,8 +532,13 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="es-CO"/>
-              <a:t>Visit motives distribution</a:t>
+              <a:t>Saturday</a:t>
             </a:r>
+            <a:r>
+              <a:rPr lang="es-CO" baseline="0"/>
+              <a:t> vs Sunday</a:t>
+            </a:r>
+            <a:endParaRPr lang="es-CO"/>
           </a:p>
         </c:rich>
       </c:tx>

</xml_diff>